<commit_message>
US98034-Update templates for uploads
</commit_message>
<xml_diff>
--- a/spreadsheet-examples/spreadsheet-libraries/SAP Cloud ALM - Library Elements Template for Configuration and Configuration Activity.xlsx
+++ b/spreadsheet-examples/spreadsheet-libraries/SAP Cloud ALM - Library Elements Template for Configuration and Configuration Activity.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3F424F5-867D-47D5-8882-7C0994F3FFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26B5111-C30C-441D-BB56-067760E4086C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library Elements" sheetId="1" r:id="rId1"/>
     <sheet name="Library &amp; Element Types" sheetId="3" r:id="rId2"/>
-    <sheet name="Categories" sheetId="4" r:id="rId3"/>
-    <sheet name="Help Portal" sheetId="5" r:id="rId4"/>
+    <sheet name="Help Portal" sheetId="5" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Library Elements'!$A$1:$O$6</definedName>
-    <definedName name="Configuration">'Library &amp; Element Types'!$B$2:$B$5</definedName>
-    <definedName name="Configuration_Activity">'Library &amp; Element Types'!$C$2:$C$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Library Elements'!$A$1:$N$6</definedName>
+    <definedName name="Configuration">'Library &amp; Element Types'!$B$2:$B$6</definedName>
+    <definedName name="Configuration_Activity">'Library &amp; Element Types'!$B$9:$B$12</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -161,7 +160,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H2" authorId="0" shapeId="0" xr:uid="{9F7F5761-177E-4631-B6B6-412ED8B717DE}">
+    <comment ref="G2" authorId="0" shapeId="0" xr:uid="{9F7F5761-177E-4631-B6B6-412ED8B717DE}">
       <text>
         <r>
           <rPr>
@@ -209,7 +208,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K3" authorId="0" shapeId="0" xr:uid="{425B44B2-FC9D-4019-9C5E-FFC88F891DBE}">
+    <comment ref="J3" authorId="0" shapeId="0" xr:uid="{425B44B2-FC9D-4019-9C5E-FFC88F891DBE}">
       <text>
         <r>
           <rPr>
@@ -238,7 +237,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="37">
   <si>
     <t>Title</t>
   </si>
@@ -258,9 +257,6 @@
     <t>Solution Component</t>
   </si>
   <si>
-    <t>Category</t>
-  </si>
-  <si>
     <t>Object</t>
   </si>
   <si>
@@ -321,12 +317,6 @@
     <t>Authorization</t>
   </si>
   <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>Available Categories</t>
-  </si>
-  <si>
     <t>Organizational Unit</t>
   </si>
   <si>
@@ -354,7 +344,10 @@
     <t>Library Types</t>
   </si>
   <si>
-    <t>Element Types</t>
+    <t>Business Role</t>
+  </si>
+  <si>
+    <t>Available Element Type</t>
   </si>
 </sst>
 </file>
@@ -481,7 +474,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -490,40 +483,15 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
+      <left style="thin">
         <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -536,28 +504,24 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -886,28 +850,27 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:BQ10"/>
-  <sheetFormatPr defaultColWidth="8.80859375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.6"/>
+  <dimension ref="A1:BP10"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="4.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.76171875" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.234375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.80859375" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="24.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.234375" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.76171875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="7.94921875" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.80859375" style="2"/>
+    <col min="1" max="1" width="21.125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="4.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.25" style="2" customWidth="1"/>
+    <col min="5" max="5" width="13.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.375" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.75" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="1" spans="1:68" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -939,20 +902,18 @@
         <v>9</v>
       </c>
       <c r="K1" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="M1" s="6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>33</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="O1" s="2"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -990,107 +951,107 @@
       <c r="AX1" s="2"/>
       <c r="AY1" s="2"/>
       <c r="AZ1" s="2"/>
-      <c r="BA1" s="2"/>
-    </row>
-    <row r="2" spans="1:69" ht="15.6" x14ac:dyDescent="0.6">
+    </row>
+    <row r="2" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2">
+        <v>5</v>
+      </c>
+      <c r="K2" s="2"/>
+    </row>
+    <row r="3" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="2">
-        <v>5</v>
-      </c>
-      <c r="L2" s="2"/>
-    </row>
-    <row r="3" spans="1:69" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="8"/>
+      <c r="H3" s="2">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="K3" s="2"/>
+    </row>
+    <row r="4" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="10"/>
-      <c r="I3" s="2">
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="L3" s="2"/>
-    </row>
-    <row r="4" spans="1:69" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A4" s="2" t="s">
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="H4" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="J4" s="8"/>
+      <c r="K4" s="2"/>
+    </row>
+    <row r="5" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="I4" s="2">
-        <v>5.2</v>
-      </c>
-      <c r="K4" s="10"/>
-      <c r="L4" s="2"/>
-    </row>
-    <row r="5" spans="1:69" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A5" s="2" t="s">
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="H5" s="2">
+        <v>5.3</v>
+      </c>
+      <c r="J5" s="8"/>
+      <c r="K5" s="2"/>
+    </row>
+    <row r="6" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="I5" s="2">
-        <v>5.3</v>
-      </c>
-      <c r="K5" s="10"/>
-      <c r="L5" s="2"/>
-    </row>
-    <row r="6" spans="1:69" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="I6" s="2">
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="H6" s="2">
         <v>5.4</v>
       </c>
-      <c r="K6" s="10"/>
-      <c r="L6" s="2"/>
-    </row>
-    <row r="7" spans="1:69" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:69" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="L8" s="2"/>
-    </row>
-    <row r="9" spans="1:69" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="L9" s="2"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="2"/>
+    </row>
+    <row r="7" spans="1:68" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K7" s="2"/>
+    </row>
+    <row r="8" spans="1:68" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K8" s="2"/>
+    </row>
+    <row r="9" spans="1:68" x14ac:dyDescent="0.25">
+      <c r="K9" s="2"/>
+      <c r="AB9" s="5"/>
       <c r="AC9" s="5"/>
       <c r="AD9" s="5"/>
       <c r="AE9" s="5"/>
@@ -1131,40 +1092,34 @@
       <c r="BN9" s="5"/>
       <c r="BO9" s="5"/>
       <c r="BP9" s="5"/>
-      <c r="BQ9" s="5"/>
-    </row>
-    <row r="10" spans="1:69" ht="15.75" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="L10" s="2"/>
+    </row>
+    <row r="10" spans="1:68" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K10" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O6" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:N6" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="E3:F6"/>
-    <mergeCell ref="K3:K6"/>
+    <mergeCell ref="J3:J6"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Choose Element Type" sqref="D2:D10" xr:uid="{87AC2146-AB06-4554-96CD-0ACC9F574EA7}">
-      <formula1>INDIRECT(SUBSTITUTE(C2," ","_"))</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Choose Library Type" prompt=" " xr:uid="{62750D3C-FA6B-4236-8F03-74C363772A60}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Choose Library Type" prompt=" " xr:uid="{EBBBD353-44CC-43AB-9EBA-DD66B41F3A07}">
           <x14:formula1>
-            <xm:f>'Library &amp; Element Types'!$B$1:$C$1</xm:f>
+            <xm:f>'Library &amp; Element Types'!$A$2:$A$12</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C20</xm:sqref>
+          <xm:sqref>C2:C1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Choose Category" prompt=" " xr:uid="{F964434D-22F3-4FB7-8F3A-6D5AEAA1F833}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Choose Element Type" xr:uid="{0F8265A2-5085-4F1E-A75E-71787550E9DA}">
           <x14:formula1>
-            <xm:f>Categories!$A$2:$A$8</xm:f>
+            <xm:f>'Library &amp; Element Types'!$B$2:$B$12</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G10</xm:sqref>
+          <xm:sqref>D2:D1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1174,143 +1129,124 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0148C08-9615-D040-B920-96C17CC67CC7}">
-  <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultColWidth="10.80859375" defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.6171875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="10.80859375" style="2"/>
+    <col min="1" max="1" width="20" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.75" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.6">
-      <c r="A1" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1" s="9" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="10"/>
+      <c r="B3" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="10"/>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="10"/>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="10"/>
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="10"/>
+      <c r="B7" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.6">
-      <c r="A2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.6">
-      <c r="A3" s="12"/>
-      <c r="C3" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.6">
-      <c r="A4" s="12"/>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.6">
-      <c r="A5" s="12"/>
-      <c r="C5" s="1" t="s">
-        <v>22</v>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="1" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:A5"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0303B768-7198-F346-AE46-E4635DF74FC2}">
-  <dimension ref="A1:A8"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
-  <cols>
-    <col min="1" max="1" width="30.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="11" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A1" s="6" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A2" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A3" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A4" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A5" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A6" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A7" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.6">
-      <c r="A8" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:A8">
-    <sortCondition ref="A2:A8"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{574F8865-6568-43EE-85C4-2FD9BB5A44FB}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A4:H4"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.6" x14ac:dyDescent="0.6"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="10.6640625" style="3"/>
+    <col min="1" max="16384" width="10.625" style="3"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A4" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="B4" s="13"/>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1325,6 +1261,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d732dc85-02c4-4698-b283-fa972b8844f9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9a63c5a5-df7a-4c5d-9f59-18edb26dfc02" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1333,7 +1280,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100549613C24315B4448A1E41B4719784FE" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5d93bc61055e9fc41fcd19f7bd54afd4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d732dc85-02c4-4698-b283-fa972b8844f9" xmlns:ns3="9a63c5a5-df7a-4c5d-9f59-18edb26dfc02" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="64abf6ef7f177d3de22be4dd574d709e" ns2:_="" ns3:_="">
     <xsd:import namespace="d732dc85-02c4-4698-b283-fa972b8844f9"/>
@@ -1534,18 +1481,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d732dc85-02c4-4698-b283-fa972b8844f9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9a63c5a5-df7a-4c5d-9f59-18edb26dfc02" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5A26520-C4EA-4E95-94B4-40DA8F7673B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d732dc85-02c4-4698-b283-fa972b8844f9"/>
+    <ds:schemaRef ds:uri="9a63c5a5-df7a-4c5d-9f59-18edb26dfc02"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{589664EC-063F-42CF-9F49-3AC2337402A9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -1553,7 +1500,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08FE90CA-7165-4041-8354-50A71455E101}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1572,17 +1519,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5A26520-C4EA-4E95-94B4-40DA8F7673B2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d732dc85-02c4-4698-b283-fa972b8844f9"/>
-    <ds:schemaRef ds:uri="9a63c5a5-df7a-4c5d-9f59-18edb26dfc02"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{0cf7ac0a-4681-4823-ab0b-04ef02c5f873}" enabled="1" method="Standard" siteId="{42f7676c-f455-423c-82f6-dc2d99791af7}" contentBits="0" removed="0"/>

</xml_diff>